<commit_message>
Feat: Add integrated Dashboard sheet with embedded chart asset
</commit_message>
<xml_diff>
--- a/Sales_Analysis_Report.xlsx
+++ b/Sales_Analysis_Report.xlsx
@@ -419,18 +419,6 @@
   </sheetPr>
   <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9297,12 +9285,6 @@
   </sheetPr>
   <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -10139,9 +10121,6 @@
   </sheetPr>
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -10168,12 +10147,6 @@
   </sheetPr>
   <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -13810,10 +13783,6 @@
   </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>